<commit_message>
Release 8 apr 2026: SMTP, viaggi UI, FK errors, DB functions
- AziendaSmtpService: salva risultati test su DB, recupera password reale
- SmtpEmailSender: timeout 30s, cert flessibile, logging, header To
- StampaBilancioViaggioDialog: modalita menu vs prefissata da DataGrid
- AnaViaggiDialog: split Create/Edit, creazione atomica con date
- AnaViaggi: auto-expand viaggio appena creato nell albero
- MovClientiViaggiService: messaggi errore FK user-friendly
- EnterpriseDataGrid: default page size 25
- fn_get_viaggi_init_data: fix nomi colonne + ORDER BY in json_agg
- fn_get_date_viaggi_with_transactions: filtra ANNULLATO e causale documento
- csproj: escludi Test*.cs e test_*.cs dalla compilazione

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inp_Excel/ana_date_viaggi.xlsx
+++ b/inp_Excel/ana_date_viaggi.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="22">
   <si>
     <t>VIAGGIO_ID_FK</t>
   </si>
@@ -178,8 +178,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:P142" totalsRowShown="0" headerRowCount="1">
-  <autoFilter ref="A1:P142"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:P144" totalsRowShown="0" headerRowCount="1">
+  <autoFilter ref="A1:P144"/>
   <tableColumns count="16">
     <tableColumn id="1" name="VIAGGIO_ID_FK"/>
     <tableColumn id="2" name="DATA_VIAGGIO_ID"/>
@@ -1271,10 +1271,10 @@
         <v>1784</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>46045</v>
+        <v>46066</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>46047</v>
+        <v>46068</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>16</v>
@@ -1294,10 +1294,14 @@
         <v>19</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>45983.3522106481</v>
-      </c>
-      <c r="O28" s="7"/>
-      <c r="P28" s="8"/>
+        <v>45983</v>
+      </c>
+      <c r="O28" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="P28" s="8" t="n">
+        <v>46053.8093518519</v>
+      </c>
     </row>
     <row r="29" customHeight="1" ht="20">
       <c r="A29" s="5" t="n">
@@ -1997,13 +2001,13 @@
         <v>1584</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>45774</v>
+        <v>46160</v>
       </c>
       <c r="D47" s="6" t="n">
-        <v>45780</v>
+        <v>46165</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F47" s="5" t="n">
         <v>1060</v>
@@ -2026,7 +2030,7 @@
         <v>19</v>
       </c>
       <c r="P47" s="8" t="n">
-        <v>45793.6937847222</v>
+        <v>46053.8084606481</v>
       </c>
     </row>
     <row r="48" customHeight="1" ht="20">
@@ -2727,25 +2731,25 @@
     </row>
     <row r="66" customHeight="1" ht="20">
       <c r="A66" s="5" t="n">
-        <v>1</v>
+        <v>901</v>
       </c>
       <c r="B66" s="5" t="n">
-        <v>24</v>
+        <v>1863</v>
       </c>
       <c r="C66" s="6" t="n">
-        <v>44324</v>
+        <v>46106</v>
       </c>
       <c r="D66" s="6" t="n">
-        <v>44325</v>
+        <v>46109</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>230</v>
+        <v>590</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>130</v>
+        <v>590</v>
       </c>
       <c r="H66" s="5"/>
       <c r="I66" s="5"/>
@@ -2753,26 +2757,26 @@
       <c r="K66" s="5"/>
       <c r="L66" s="7"/>
       <c r="M66" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="N66" s="8" t="n">
-        <v>44420.5177546296</v>
+        <v>46053.8152199074</v>
       </c>
       <c r="O66" s="7"/>
       <c r="P66" s="8"/>
     </row>
     <row r="67" customHeight="1" ht="20">
       <c r="A67" s="5" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="B67" s="5" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C67" s="6" t="n">
-        <v>43995</v>
+        <v>44324</v>
       </c>
       <c r="D67" s="6" t="n">
-        <v>43996</v>
+        <v>44325</v>
       </c>
       <c r="E67" s="7" t="s">
         <v>18</v>
@@ -2792,7 +2796,7 @@
         <v>17</v>
       </c>
       <c r="N67" s="8" t="n">
-        <v>44420.5183796296</v>
+        <v>44420.5177546296</v>
       </c>
       <c r="O67" s="7"/>
       <c r="P67" s="8"/>
@@ -2802,13 +2806,13 @@
         <v>22</v>
       </c>
       <c r="B68" s="5" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C68" s="6" t="n">
-        <v>44121</v>
+        <v>43995</v>
       </c>
       <c r="D68" s="6" t="n">
-        <v>44122</v>
+        <v>43996</v>
       </c>
       <c r="E68" s="7" t="s">
         <v>18</v>
@@ -2828,32 +2832,32 @@
         <v>17</v>
       </c>
       <c r="N68" s="8" t="n">
-        <v>44420.5187268519</v>
+        <v>44420.5183796296</v>
       </c>
       <c r="O68" s="7"/>
       <c r="P68" s="8"/>
     </row>
     <row r="69" customHeight="1" ht="20">
       <c r="A69" s="5" t="n">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="B69" s="5" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="C69" s="6" t="n">
-        <v>44149</v>
+        <v>44121</v>
       </c>
       <c r="D69" s="6" t="n">
-        <v>44149</v>
+        <v>44122</v>
       </c>
       <c r="E69" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F69" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="G69" s="5" t="n">
         <v>130</v>
-      </c>
-      <c r="G69" s="5" t="n">
-        <v>30</v>
       </c>
       <c r="H69" s="5"/>
       <c r="I69" s="5"/>
@@ -2864,26 +2868,26 @@
         <v>17</v>
       </c>
       <c r="N69" s="8" t="n">
-        <v>44446.5248032407</v>
+        <v>44420.5187268519</v>
       </c>
       <c r="O69" s="7"/>
       <c r="P69" s="8"/>
     </row>
     <row r="70" customHeight="1" ht="20">
       <c r="A70" s="5" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B70" s="5" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="C70" s="6" t="n">
-        <v>44492</v>
+        <v>44149</v>
       </c>
       <c r="D70" s="6" t="n">
-        <v>44492</v>
+        <v>44149</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F70" s="5" t="n">
         <v>130</v>
@@ -2900,36 +2904,32 @@
         <v>17</v>
       </c>
       <c r="N70" s="8" t="n">
-        <v>44446</v>
-      </c>
-      <c r="O70" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P70" s="8" t="n">
-        <v>44785.5593287037</v>
-      </c>
+        <v>44446.5248032407</v>
+      </c>
+      <c r="O70" s="7"/>
+      <c r="P70" s="8"/>
     </row>
     <row r="71" customHeight="1" ht="20">
       <c r="A71" s="5" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B71" s="5" t="n">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="C71" s="6" t="n">
-        <v>44133</v>
+        <v>44492</v>
       </c>
       <c r="D71" s="6" t="n">
-        <v>44136</v>
+        <v>44492</v>
       </c>
       <c r="E71" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>520</v>
+        <v>130</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>280</v>
+        <v>30</v>
       </c>
       <c r="H71" s="5"/>
       <c r="I71" s="5"/>
@@ -2946,30 +2946,30 @@
         <v>17</v>
       </c>
       <c r="P71" s="8" t="n">
-        <v>44847.4125231481</v>
+        <v>44785.5593287037</v>
       </c>
     </row>
     <row r="72" customHeight="1" ht="20">
       <c r="A72" s="5" t="n">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="B72" s="5" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="C72" s="6" t="n">
-        <v>43690</v>
+        <v>44133</v>
       </c>
       <c r="D72" s="6" t="n">
-        <v>43697</v>
+        <v>44136</v>
       </c>
       <c r="E72" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>780</v>
+        <v>520</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>560</v>
+        <v>280</v>
       </c>
       <c r="H72" s="5"/>
       <c r="I72" s="5"/>
@@ -2980,32 +2980,36 @@
         <v>17</v>
       </c>
       <c r="N72" s="8" t="n">
-        <v>44446.5365856481</v>
-      </c>
-      <c r="O72" s="7"/>
-      <c r="P72" s="8"/>
+        <v>44446</v>
+      </c>
+      <c r="O72" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P72" s="8" t="n">
+        <v>44847.4125231481</v>
+      </c>
     </row>
     <row r="73" customHeight="1" ht="20">
       <c r="A73" s="5" t="n">
         <v>27</v>
       </c>
       <c r="B73" s="5" t="n">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C73" s="6" t="n">
-        <v>44380</v>
+        <v>43690</v>
       </c>
       <c r="D73" s="6" t="n">
-        <v>44386</v>
+        <v>43697</v>
       </c>
       <c r="E73" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>820</v>
+        <v>780</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>590</v>
+        <v>560</v>
       </c>
       <c r="H73" s="5"/>
       <c r="I73" s="5"/>
@@ -3016,32 +3020,32 @@
         <v>17</v>
       </c>
       <c r="N73" s="8" t="n">
-        <v>44446.5373958333</v>
+        <v>44446.5365856481</v>
       </c>
       <c r="O73" s="7"/>
       <c r="P73" s="8"/>
     </row>
     <row r="74" customHeight="1" ht="20">
       <c r="A74" s="5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B74" s="5" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C74" s="6" t="n">
-        <v>43932</v>
+        <v>44380</v>
       </c>
       <c r="D74" s="6" t="n">
-        <v>43938</v>
+        <v>44386</v>
       </c>
       <c r="E74" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>890</v>
+        <v>820</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>580</v>
+        <v>590</v>
       </c>
       <c r="H74" s="5"/>
       <c r="I74" s="5"/>
@@ -3052,7 +3056,7 @@
         <v>17</v>
       </c>
       <c r="N74" s="8" t="n">
-        <v>44446.5383217593</v>
+        <v>44446.5373958333</v>
       </c>
       <c r="O74" s="7"/>
       <c r="P74" s="8"/>
@@ -3062,22 +3066,22 @@
         <v>25</v>
       </c>
       <c r="B75" s="5" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C75" s="6" t="n">
-        <v>44380</v>
+        <v>43932</v>
       </c>
       <c r="D75" s="6" t="n">
-        <v>44386</v>
+        <v>43938</v>
       </c>
       <c r="E75" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F75" s="5" t="n">
         <v>890</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>590</v>
+        <v>580</v>
       </c>
       <c r="H75" s="5"/>
       <c r="I75" s="5"/>
@@ -3088,32 +3092,32 @@
         <v>17</v>
       </c>
       <c r="N75" s="8" t="n">
-        <v>44446.5391898148</v>
+        <v>44446.5383217593</v>
       </c>
       <c r="O75" s="7"/>
       <c r="P75" s="8"/>
     </row>
     <row r="76" customHeight="1" ht="20">
       <c r="A76" s="5" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="B76" s="5" t="n">
-        <v>182</v>
+        <v>78</v>
       </c>
       <c r="C76" s="6" t="n">
-        <v>44611</v>
+        <v>44380</v>
       </c>
       <c r="D76" s="6" t="n">
-        <v>44612</v>
+        <v>44386</v>
       </c>
       <c r="E76" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>245</v>
+        <v>890</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>140</v>
+        <v>590</v>
       </c>
       <c r="H76" s="5"/>
       <c r="I76" s="5"/>
@@ -3124,36 +3128,32 @@
         <v>17</v>
       </c>
       <c r="N76" s="8" t="n">
-        <v>44603</v>
-      </c>
-      <c r="O76" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P76" s="8" t="n">
-        <v>44620.6170717593</v>
-      </c>
+        <v>44446.5391898148</v>
+      </c>
+      <c r="O76" s="7"/>
+      <c r="P76" s="8"/>
     </row>
     <row r="77" customHeight="1" ht="20">
       <c r="A77" s="5" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B77" s="5" t="n">
-        <v>302</v>
+        <v>182</v>
       </c>
       <c r="C77" s="6" t="n">
-        <v>44786</v>
+        <v>44611</v>
       </c>
       <c r="D77" s="6" t="n">
-        <v>44797</v>
+        <v>44612</v>
       </c>
       <c r="E77" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>1440</v>
+        <v>245</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>990</v>
+        <v>140</v>
       </c>
       <c r="H77" s="5"/>
       <c r="I77" s="5"/>
@@ -3164,32 +3164,36 @@
         <v>17</v>
       </c>
       <c r="N77" s="8" t="n">
-        <v>44655.6645833333</v>
-      </c>
-      <c r="O77" s="7"/>
-      <c r="P77" s="8"/>
+        <v>44603</v>
+      </c>
+      <c r="O77" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P77" s="8" t="n">
+        <v>44620.6170717593</v>
+      </c>
     </row>
     <row r="78" customHeight="1" ht="20">
       <c r="A78" s="5" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B78" s="5" t="n">
-        <v>363</v>
+        <v>302</v>
       </c>
       <c r="C78" s="6" t="n">
-        <v>44737</v>
+        <v>44786</v>
       </c>
       <c r="D78" s="6" t="n">
-        <v>44743</v>
+        <v>44797</v>
       </c>
       <c r="E78" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F78" s="5" t="n">
-        <v>890</v>
+        <v>1440</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>590</v>
+        <v>990</v>
       </c>
       <c r="H78" s="5"/>
       <c r="I78" s="5"/>
@@ -3200,40 +3204,34 @@
         <v>17</v>
       </c>
       <c r="N78" s="8" t="n">
-        <v>44679</v>
-      </c>
-      <c r="O78" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P78" s="8" t="n">
-        <v>44745.8054282407</v>
-      </c>
+        <v>44655.6645833333</v>
+      </c>
+      <c r="O78" s="7"/>
+      <c r="P78" s="8"/>
     </row>
     <row r="79" customHeight="1" ht="20">
       <c r="A79" s="5" t="n">
-        <v>141</v>
+        <v>27</v>
       </c>
       <c r="B79" s="5" t="n">
-        <v>462</v>
+        <v>363</v>
       </c>
       <c r="C79" s="6" t="n">
-        <v>44898</v>
+        <v>44737</v>
       </c>
       <c r="D79" s="6" t="n">
-        <v>44907</v>
+        <v>44743</v>
       </c>
       <c r="E79" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F79" s="5" t="n">
-        <v>1600</v>
+        <v>890</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>1350</v>
-      </c>
-      <c r="H79" s="5" t="n">
-        <v>1550</v>
-      </c>
+        <v>590</v>
+      </c>
+      <c r="H79" s="5"/>
       <c r="I79" s="5"/>
       <c r="J79" s="5"/>
       <c r="K79" s="5"/>
@@ -3242,38 +3240,40 @@
         <v>17</v>
       </c>
       <c r="N79" s="8" t="n">
-        <v>44791</v>
+        <v>44679</v>
       </c>
       <c r="O79" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P79" s="8" t="n">
-        <v>44915.6469675926</v>
+        <v>44745.8054282407</v>
       </c>
     </row>
     <row r="80" customHeight="1" ht="20">
       <c r="A80" s="5" t="n">
-        <v>201</v>
+        <v>141</v>
       </c>
       <c r="B80" s="5" t="n">
-        <v>522</v>
+        <v>462</v>
       </c>
       <c r="C80" s="6" t="n">
-        <v>44856</v>
+        <v>44898</v>
       </c>
       <c r="D80" s="6" t="n">
-        <v>44857</v>
+        <v>44907</v>
       </c>
       <c r="E80" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F80" s="5" t="n">
-        <v>245</v>
+        <v>1600</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>140</v>
-      </c>
-      <c r="H80" s="5"/>
+        <v>1350</v>
+      </c>
+      <c r="H80" s="5" t="n">
+        <v>1550</v>
+      </c>
       <c r="I80" s="5"/>
       <c r="J80" s="5"/>
       <c r="K80" s="5"/>
@@ -3282,36 +3282,36 @@
         <v>17</v>
       </c>
       <c r="N80" s="8" t="n">
-        <v>44834</v>
+        <v>44791</v>
       </c>
       <c r="O80" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P80" s="8" t="n">
-        <v>44837.3615972222</v>
+        <v>44915.6469675926</v>
       </c>
     </row>
     <row r="81" customHeight="1" ht="20">
       <c r="A81" s="5" t="n">
-        <v>101</v>
+        <v>201</v>
       </c>
       <c r="B81" s="5" t="n">
-        <v>742</v>
+        <v>522</v>
       </c>
       <c r="C81" s="6" t="n">
-        <v>45010</v>
+        <v>44856</v>
       </c>
       <c r="D81" s="6" t="n">
-        <v>45011</v>
+        <v>44857</v>
       </c>
       <c r="E81" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F81" s="5" t="n">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="G81" s="5" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="H81" s="5"/>
       <c r="I81" s="5"/>
@@ -3322,36 +3322,36 @@
         <v>17</v>
       </c>
       <c r="N81" s="8" t="n">
-        <v>44994</v>
+        <v>44834</v>
       </c>
       <c r="O81" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P81" s="8" t="n">
-        <v>45012.3928240741</v>
+        <v>44837.3615972222</v>
       </c>
     </row>
     <row r="82" customHeight="1" ht="20">
       <c r="A82" s="5" t="n">
-        <v>23</v>
+        <v>101</v>
       </c>
       <c r="B82" s="5" t="n">
-        <v>782</v>
+        <v>742</v>
       </c>
       <c r="C82" s="6" t="n">
-        <v>45115</v>
+        <v>45010</v>
       </c>
       <c r="D82" s="6" t="n">
-        <v>45127</v>
+        <v>45011</v>
       </c>
       <c r="E82" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F82" s="5" t="n">
-        <v>1490</v>
+        <v>250</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>995</v>
+        <v>150</v>
       </c>
       <c r="H82" s="5"/>
       <c r="I82" s="5"/>
@@ -3362,32 +3362,36 @@
         <v>17</v>
       </c>
       <c r="N82" s="8" t="n">
-        <v>45013.6681597222</v>
-      </c>
-      <c r="O82" s="7"/>
-      <c r="P82" s="8"/>
+        <v>44994</v>
+      </c>
+      <c r="O82" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P82" s="8" t="n">
+        <v>45012.3928240741</v>
+      </c>
     </row>
     <row r="83" customHeight="1" ht="20">
       <c r="A83" s="5" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="B83" s="5" t="n">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C83" s="6" t="n">
-        <v>45101</v>
+        <v>45115</v>
       </c>
       <c r="D83" s="6" t="n">
-        <v>45108</v>
+        <v>45127</v>
       </c>
       <c r="E83" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F83" s="5" t="n">
-        <v>1100</v>
+        <v>1490</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>710</v>
+        <v>995</v>
       </c>
       <c r="H83" s="5"/>
       <c r="I83" s="5"/>
@@ -3398,32 +3402,32 @@
         <v>17</v>
       </c>
       <c r="N83" s="8" t="n">
-        <v>45013.6687037037</v>
+        <v>45013.6681597222</v>
       </c>
       <c r="O83" s="7"/>
       <c r="P83" s="8"/>
     </row>
     <row r="84" customHeight="1" ht="20">
       <c r="A84" s="5" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B84" s="5" t="n">
-        <v>942</v>
+        <v>783</v>
       </c>
       <c r="C84" s="6" t="n">
-        <v>45107</v>
+        <v>45101</v>
       </c>
       <c r="D84" s="6" t="n">
-        <v>45109</v>
+        <v>45108</v>
       </c>
       <c r="E84" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F84" s="5" t="n">
-        <v>180</v>
+        <v>1100</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>100</v>
+        <v>710</v>
       </c>
       <c r="H84" s="5"/>
       <c r="I84" s="5"/>
@@ -3434,36 +3438,32 @@
         <v>17</v>
       </c>
       <c r="N84" s="8" t="n">
-        <v>45080</v>
-      </c>
-      <c r="O84" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P84" s="8" t="n">
-        <v>45111.2536921296</v>
-      </c>
+        <v>45013.6687037037</v>
+      </c>
+      <c r="O84" s="7"/>
+      <c r="P84" s="8"/>
     </row>
     <row r="85" customHeight="1" ht="20">
       <c r="A85" s="5" t="n">
-        <v>381</v>
+        <v>26</v>
       </c>
       <c r="B85" s="5" t="n">
-        <v>962</v>
+        <v>942</v>
       </c>
       <c r="C85" s="6" t="n">
-        <v>45110</v>
+        <v>45107</v>
       </c>
       <c r="D85" s="6" t="n">
-        <v>45111</v>
+        <v>45109</v>
       </c>
       <c r="E85" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F85" s="5" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="G85" s="5" t="n">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="H85" s="5"/>
       <c r="I85" s="5"/>
@@ -3474,13 +3474,13 @@
         <v>17</v>
       </c>
       <c r="N85" s="8" t="n">
-        <v>45082</v>
+        <v>45080</v>
       </c>
       <c r="O85" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P85" s="8" t="n">
-        <v>45111.2538310185</v>
+        <v>45111.2536921296</v>
       </c>
     </row>
     <row r="86" customHeight="1" ht="20">
@@ -3488,22 +3488,22 @@
         <v>381</v>
       </c>
       <c r="B86" s="5" t="n">
-        <v>1082</v>
+        <v>962</v>
       </c>
       <c r="C86" s="6" t="n">
-        <v>45177</v>
+        <v>45110</v>
       </c>
       <c r="D86" s="6" t="n">
-        <v>45179</v>
+        <v>45111</v>
       </c>
       <c r="E86" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F86" s="5" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H86" s="5"/>
       <c r="I86" s="5"/>
@@ -3514,36 +3514,36 @@
         <v>17</v>
       </c>
       <c r="N86" s="8" t="n">
-        <v>45173</v>
+        <v>45082</v>
       </c>
       <c r="O86" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P86" s="8" t="n">
-        <v>45173.6145601852</v>
+        <v>45111.2538310185</v>
       </c>
     </row>
     <row r="87" customHeight="1" ht="20">
       <c r="A87" s="5" t="n">
-        <v>301</v>
+        <v>381</v>
       </c>
       <c r="B87" s="5" t="n">
-        <v>1122</v>
+        <v>1082</v>
       </c>
       <c r="C87" s="6" t="n">
-        <v>45268</v>
+        <v>45177</v>
       </c>
       <c r="D87" s="6" t="n">
-        <v>45270</v>
+        <v>45179</v>
       </c>
       <c r="E87" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F87" s="5" t="n">
-        <v>370</v>
+        <v>500</v>
       </c>
       <c r="G87" s="5" t="n">
-        <v>145</v>
+        <v>500</v>
       </c>
       <c r="H87" s="5"/>
       <c r="I87" s="5"/>
@@ -3554,36 +3554,36 @@
         <v>17</v>
       </c>
       <c r="N87" s="8" t="n">
-        <v>45205</v>
+        <v>45173</v>
       </c>
       <c r="O87" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P87" s="8" t="n">
-        <v>45267.4084143519</v>
+        <v>45173.6145601852</v>
       </c>
     </row>
     <row r="88" customHeight="1" ht="20">
       <c r="A88" s="5" t="n">
-        <v>81</v>
+        <v>301</v>
       </c>
       <c r="B88" s="5" t="n">
-        <v>1162</v>
+        <v>1122</v>
       </c>
       <c r="C88" s="6" t="n">
-        <v>45318</v>
+        <v>45268</v>
       </c>
       <c r="D88" s="6" t="n">
-        <v>45319</v>
+        <v>45270</v>
       </c>
       <c r="E88" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F88" s="5" t="n">
-        <v>250</v>
+        <v>370</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="H88" s="5"/>
       <c r="I88" s="5"/>
@@ -3594,36 +3594,36 @@
         <v>17</v>
       </c>
       <c r="N88" s="8" t="n">
-        <v>45274</v>
+        <v>45205</v>
       </c>
       <c r="O88" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P88" s="8" t="n">
-        <v>45320.4609837963</v>
+        <v>45267.4084143519</v>
       </c>
     </row>
     <row r="89" customHeight="1" ht="20">
       <c r="A89" s="5" t="n">
-        <v>441</v>
+        <v>81</v>
       </c>
       <c r="B89" s="5" t="n">
-        <v>1182</v>
+        <v>1162</v>
       </c>
       <c r="C89" s="6" t="n">
-        <v>45290</v>
+        <v>45318</v>
       </c>
       <c r="D89" s="6" t="n">
-        <v>45295</v>
+        <v>45319</v>
       </c>
       <c r="E89" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>860</v>
+        <v>250</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>660</v>
+        <v>150</v>
       </c>
       <c r="H89" s="5"/>
       <c r="I89" s="5"/>
@@ -3634,36 +3634,36 @@
         <v>17</v>
       </c>
       <c r="N89" s="8" t="n">
-        <v>45277</v>
+        <v>45274</v>
       </c>
       <c r="O89" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P89" s="8" t="n">
-        <v>45285.4578009259</v>
+        <v>45320.4609837963</v>
       </c>
     </row>
     <row r="90" customHeight="1" ht="20">
       <c r="A90" s="5" t="n">
-        <v>261</v>
+        <v>441</v>
       </c>
       <c r="B90" s="5" t="n">
-        <v>1202</v>
+        <v>1182</v>
       </c>
       <c r="C90" s="6" t="n">
-        <v>45366</v>
+        <v>45290</v>
       </c>
       <c r="D90" s="6" t="n">
-        <v>45368</v>
+        <v>45295</v>
       </c>
       <c r="E90" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>385</v>
+        <v>860</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>240</v>
+        <v>660</v>
       </c>
       <c r="H90" s="5"/>
       <c r="I90" s="5"/>
@@ -3674,36 +3674,36 @@
         <v>17</v>
       </c>
       <c r="N90" s="8" t="n">
-        <v>45280</v>
+        <v>45277</v>
       </c>
       <c r="O90" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P90" s="8" t="n">
-        <v>45419.522962963</v>
+        <v>45285.4578009259</v>
       </c>
     </row>
     <row r="91" customHeight="1" ht="20">
       <c r="A91" s="5" t="n">
-        <v>181</v>
+        <v>261</v>
       </c>
       <c r="B91" s="5" t="n">
-        <v>1262</v>
+        <v>1202</v>
       </c>
       <c r="C91" s="6" t="n">
-        <v>45339</v>
+        <v>45366</v>
       </c>
       <c r="D91" s="6" t="n">
-        <v>45340</v>
+        <v>45368</v>
       </c>
       <c r="E91" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F91" s="5" t="n">
-        <v>250</v>
+        <v>385</v>
       </c>
       <c r="G91" s="5" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="H91" s="5"/>
       <c r="I91" s="5"/>
@@ -3714,36 +3714,36 @@
         <v>17</v>
       </c>
       <c r="N91" s="8" t="n">
-        <v>45303</v>
+        <v>45280</v>
       </c>
       <c r="O91" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P91" s="8" t="n">
-        <v>45343.4145486111</v>
+        <v>45419.522962963</v>
       </c>
     </row>
     <row r="92" customHeight="1" ht="20">
       <c r="A92" s="5" t="n">
-        <v>27</v>
+        <v>181</v>
       </c>
       <c r="B92" s="5" t="n">
-        <v>1342</v>
+        <v>1262</v>
       </c>
       <c r="C92" s="6" t="n">
-        <v>45444</v>
+        <v>45339</v>
       </c>
       <c r="D92" s="6" t="n">
-        <v>45451</v>
+        <v>45340</v>
       </c>
       <c r="E92" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F92" s="5" t="n">
-        <v>940</v>
+        <v>250</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>590</v>
+        <v>150</v>
       </c>
       <c r="H92" s="5"/>
       <c r="I92" s="5"/>
@@ -3754,32 +3754,36 @@
         <v>17</v>
       </c>
       <c r="N92" s="8" t="n">
-        <v>45313.4136458333</v>
-      </c>
-      <c r="O92" s="7"/>
-      <c r="P92" s="8"/>
+        <v>45303</v>
+      </c>
+      <c r="O92" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P92" s="8" t="n">
+        <v>45343.4145486111</v>
+      </c>
     </row>
     <row r="93" customHeight="1" ht="20">
       <c r="A93" s="5" t="n">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="B93" s="5" t="n">
-        <v>1403</v>
+        <v>1342</v>
       </c>
       <c r="C93" s="6" t="n">
+        <v>45444</v>
+      </c>
+      <c r="D93" s="6" t="n">
         <v>45451</v>
-      </c>
-      <c r="D93" s="6" t="n">
-        <v>45459</v>
       </c>
       <c r="E93" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F93" s="5" t="n">
-        <v>990</v>
+        <v>940</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>690</v>
+        <v>590</v>
       </c>
       <c r="H93" s="5"/>
       <c r="I93" s="5"/>
@@ -3790,32 +3794,32 @@
         <v>17</v>
       </c>
       <c r="N93" s="8" t="n">
-        <v>45348.3647453704</v>
+        <v>45313.4136458333</v>
       </c>
       <c r="O93" s="7"/>
       <c r="P93" s="8"/>
     </row>
     <row r="94" customHeight="1" ht="20">
       <c r="A94" s="5" t="n">
-        <v>321</v>
+        <v>41</v>
       </c>
       <c r="B94" s="5" t="n">
-        <v>1444</v>
+        <v>1403</v>
       </c>
       <c r="C94" s="6" t="n">
-        <v>45464</v>
+        <v>45451</v>
       </c>
       <c r="D94" s="6" t="n">
-        <v>45478</v>
+        <v>45459</v>
       </c>
       <c r="E94" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F94" s="5" t="n">
-        <v>1650</v>
+        <v>990</v>
       </c>
       <c r="G94" s="5" t="n">
-        <v>1100</v>
+        <v>690</v>
       </c>
       <c r="H94" s="5"/>
       <c r="I94" s="5"/>
@@ -3826,32 +3830,32 @@
         <v>17</v>
       </c>
       <c r="N94" s="8" t="n">
-        <v>45405.5582175926</v>
+        <v>45348.3647453704</v>
       </c>
       <c r="O94" s="7"/>
       <c r="P94" s="8"/>
     </row>
     <row r="95" customHeight="1" ht="20">
       <c r="A95" s="5" t="n">
-        <v>622</v>
+        <v>321</v>
       </c>
       <c r="B95" s="5" t="n">
-        <v>1583</v>
+        <v>1444</v>
       </c>
       <c r="C95" s="6" t="n">
-        <v>45767</v>
+        <v>45464</v>
       </c>
       <c r="D95" s="6" t="n">
-        <v>45772</v>
+        <v>45478</v>
       </c>
       <c r="E95" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F95" s="5" t="n">
-        <v>790</v>
+        <v>1650</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>790</v>
+        <v>1100</v>
       </c>
       <c r="H95" s="5"/>
       <c r="I95" s="5"/>
@@ -3859,39 +3863,35 @@
       <c r="K95" s="5"/>
       <c r="L95" s="7"/>
       <c r="M95" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="N95" s="8" t="n">
-        <v>45700</v>
-      </c>
-      <c r="O95" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="P95" s="8" t="n">
-        <v>45793.6939930556</v>
-      </c>
+        <v>45405.5582175926</v>
+      </c>
+      <c r="O95" s="7"/>
+      <c r="P95" s="8"/>
     </row>
     <row r="96" customHeight="1" ht="20">
       <c r="A96" s="5" t="n">
-        <v>861</v>
+        <v>622</v>
       </c>
       <c r="B96" s="5" t="n">
-        <v>1823</v>
+        <v>1583</v>
       </c>
       <c r="C96" s="6" t="n">
-        <v>46122</v>
+        <v>46114</v>
       </c>
       <c r="D96" s="6" t="n">
-        <v>46132</v>
+        <v>46118</v>
       </c>
       <c r="E96" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F96" s="5" t="n">
-        <v>2290</v>
+        <v>760</v>
       </c>
       <c r="G96" s="5" t="n">
-        <v>2290</v>
+        <v>770</v>
       </c>
       <c r="H96" s="5"/>
       <c r="I96" s="5"/>
@@ -3902,32 +3902,36 @@
         <v>19</v>
       </c>
       <c r="N96" s="8" t="n">
-        <v>46031.3055439815</v>
-      </c>
-      <c r="O96" s="7"/>
-      <c r="P96" s="8"/>
+        <v>45700</v>
+      </c>
+      <c r="O96" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="P96" s="8" t="n">
+        <v>46047.6481018519</v>
+      </c>
     </row>
     <row r="97" customHeight="1" ht="20">
       <c r="A97" s="5" t="n">
-        <v>681</v>
+        <v>861</v>
       </c>
       <c r="B97" s="5" t="n">
-        <v>1647</v>
+        <v>1823</v>
       </c>
       <c r="C97" s="6" t="n">
-        <v>46138</v>
+        <v>46122</v>
       </c>
       <c r="D97" s="6" t="n">
-        <v>46144</v>
+        <v>46132</v>
       </c>
       <c r="E97" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F97" s="5" t="n">
-        <v>1160</v>
+        <v>2290</v>
       </c>
       <c r="G97" s="5" t="n">
-        <v>1160</v>
+        <v>2290</v>
       </c>
       <c r="H97" s="5"/>
       <c r="I97" s="5"/>
@@ -3938,36 +3942,32 @@
         <v>19</v>
       </c>
       <c r="N97" s="8" t="n">
-        <v>45793</v>
-      </c>
-      <c r="O97" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="P97" s="8" t="n">
-        <v>45958.4886226852</v>
-      </c>
+        <v>46031.3055439815</v>
+      </c>
+      <c r="O97" s="7"/>
+      <c r="P97" s="8"/>
     </row>
     <row r="98" customHeight="1" ht="20">
       <c r="A98" s="5" t="n">
-        <v>762</v>
+        <v>681</v>
       </c>
       <c r="B98" s="5" t="n">
-        <v>1724</v>
+        <v>1647</v>
       </c>
       <c r="C98" s="6" t="n">
-        <v>46021</v>
+        <v>46138</v>
       </c>
       <c r="D98" s="6" t="n">
-        <v>46026</v>
+        <v>46144</v>
       </c>
       <c r="E98" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F98" s="5" t="n">
-        <v>990</v>
+        <v>1160</v>
       </c>
       <c r="G98" s="5" t="n">
-        <v>990</v>
+        <v>1160</v>
       </c>
       <c r="H98" s="5"/>
       <c r="I98" s="5"/>
@@ -3978,27 +3978,27 @@
         <v>19</v>
       </c>
       <c r="N98" s="8" t="n">
-        <v>45963</v>
+        <v>45793</v>
       </c>
       <c r="O98" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P98" s="8" t="n">
-        <v>46030.6411574074</v>
+        <v>45958.4886226852</v>
       </c>
     </row>
     <row r="99" customHeight="1" ht="20">
       <c r="A99" s="5" t="n">
-        <v>621</v>
+        <v>762</v>
       </c>
       <c r="B99" s="5" t="n">
-        <v>1683</v>
+        <v>1724</v>
       </c>
       <c r="C99" s="6" t="n">
-        <v>45950</v>
+        <v>46021</v>
       </c>
       <c r="D99" s="6" t="n">
-        <v>45955</v>
+        <v>46026</v>
       </c>
       <c r="E99" s="7" t="s">
         <v>18</v>
@@ -4018,36 +4018,36 @@
         <v>19</v>
       </c>
       <c r="N99" s="8" t="n">
-        <v>45908</v>
+        <v>45963</v>
       </c>
       <c r="O99" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="P99" s="8" t="n">
-        <v>45951.6467939815</v>
+        <v>46030.6411574074</v>
       </c>
     </row>
     <row r="100" customHeight="1" ht="20">
       <c r="A100" s="5" t="n">
-        <v>781</v>
+        <v>621</v>
       </c>
       <c r="B100" s="5" t="n">
-        <v>1743</v>
+        <v>1683</v>
       </c>
       <c r="C100" s="6" t="n">
-        <v>46020</v>
+        <v>45950</v>
       </c>
       <c r="D100" s="6" t="n">
-        <v>46025</v>
+        <v>45955</v>
       </c>
       <c r="E100" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F100" s="5" t="n">
-        <v>1</v>
+        <v>990</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>1</v>
+        <v>990</v>
       </c>
       <c r="H100" s="5"/>
       <c r="I100" s="5"/>
@@ -4058,36 +4058,36 @@
         <v>19</v>
       </c>
       <c r="N100" s="8" t="n">
-        <v>45964</v>
+        <v>45908</v>
       </c>
       <c r="O100" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="P100" s="8" t="n">
-        <v>46030.6409490741</v>
+        <v>45951.6467939815</v>
       </c>
     </row>
     <row r="101" customHeight="1" ht="20">
       <c r="A101" s="5" t="n">
-        <v>801</v>
+        <v>781</v>
       </c>
       <c r="B101" s="5" t="n">
-        <v>1763</v>
+        <v>1743</v>
       </c>
       <c r="C101" s="6" t="n">
-        <v>46137</v>
+        <v>46020</v>
       </c>
       <c r="D101" s="6" t="n">
-        <v>46143</v>
+        <v>46025</v>
       </c>
       <c r="E101" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F101" s="5" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="H101" s="5"/>
       <c r="I101" s="5"/>
@@ -4098,32 +4098,36 @@
         <v>19</v>
       </c>
       <c r="N101" s="8" t="n">
-        <v>45981.7479166667</v>
-      </c>
-      <c r="O101" s="7"/>
-      <c r="P101" s="8"/>
+        <v>45964</v>
+      </c>
+      <c r="O101" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P101" s="8" t="n">
+        <v>46030.6409490741</v>
+      </c>
     </row>
     <row r="102" customHeight="1" ht="20">
       <c r="A102" s="5" t="n">
-        <v>1</v>
+        <v>801</v>
       </c>
       <c r="B102" s="5" t="n">
-        <v>1</v>
+        <v>1763</v>
       </c>
       <c r="C102" s="6" t="n">
-        <v>43505</v>
+        <v>46137</v>
       </c>
       <c r="D102" s="6" t="n">
-        <v>43506</v>
+        <v>46143</v>
       </c>
       <c r="E102" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>230</v>
+        <v>1000</v>
       </c>
       <c r="G102" s="5" t="n">
-        <v>130</v>
+        <v>1000</v>
       </c>
       <c r="H102" s="5"/>
       <c r="I102" s="5"/>
@@ -4131,39 +4135,35 @@
       <c r="K102" s="5"/>
       <c r="L102" s="7"/>
       <c r="M102" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="N102" s="8" t="n">
-        <v>44420</v>
-      </c>
-      <c r="O102" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P102" s="8" t="n">
-        <v>44853.7957060185</v>
-      </c>
+        <v>45981.7479166667</v>
+      </c>
+      <c r="O102" s="7"/>
+      <c r="P102" s="8"/>
     </row>
     <row r="103" customHeight="1" ht="20">
       <c r="A103" s="5" t="n">
-        <v>54</v>
+        <v>881</v>
       </c>
       <c r="B103" s="5" t="n">
-        <v>42</v>
+        <v>1843</v>
       </c>
       <c r="C103" s="6" t="n">
-        <v>44345</v>
+        <v>46104</v>
       </c>
       <c r="D103" s="6" t="n">
-        <v>44346</v>
+        <v>46108</v>
       </c>
       <c r="E103" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F103" s="5" t="n">
-        <v>230</v>
+        <v>660</v>
       </c>
       <c r="G103" s="5" t="n">
-        <v>130</v>
+        <v>660</v>
       </c>
       <c r="H103" s="5"/>
       <c r="I103" s="5"/>
@@ -4171,26 +4171,26 @@
       <c r="K103" s="5"/>
       <c r="L103" s="7"/>
       <c r="M103" s="7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="N103" s="8" t="n">
-        <v>44445.5079513889</v>
+        <v>46049.8521064815</v>
       </c>
       <c r="O103" s="7"/>
       <c r="P103" s="8"/>
     </row>
     <row r="104" customHeight="1" ht="20">
       <c r="A104" s="5" t="n">
-        <v>54</v>
+        <v>1</v>
       </c>
       <c r="B104" s="5" t="n">
-        <v>43</v>
+        <v>1</v>
       </c>
       <c r="C104" s="6" t="n">
-        <v>44464</v>
+        <v>43505</v>
       </c>
       <c r="D104" s="6" t="n">
-        <v>44465</v>
+        <v>43506</v>
       </c>
       <c r="E104" s="7" t="s">
         <v>18</v>
@@ -4210,27 +4210,27 @@
         <v>17</v>
       </c>
       <c r="N104" s="8" t="n">
-        <v>44445</v>
+        <v>44420</v>
       </c>
       <c r="O104" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P104" s="8" t="n">
-        <v>44764.5626388889</v>
+        <v>44853.7957060185</v>
       </c>
     </row>
     <row r="105" customHeight="1" ht="20">
       <c r="A105" s="5" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B105" s="5" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C105" s="6" t="n">
-        <v>44474</v>
+        <v>44345</v>
       </c>
       <c r="D105" s="6" t="n">
-        <v>44475</v>
+        <v>44346</v>
       </c>
       <c r="E105" s="7" t="s">
         <v>16</v>
@@ -4250,27 +4250,23 @@
         <v>17</v>
       </c>
       <c r="N105" s="8" t="n">
-        <v>44446.2805902778</v>
-      </c>
-      <c r="O105" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P105" s="8" t="n">
-        <v>44586.645775463</v>
-      </c>
+        <v>44445.5079513889</v>
+      </c>
+      <c r="O105" s="7"/>
+      <c r="P105" s="8"/>
     </row>
     <row r="106" customHeight="1" ht="20">
       <c r="A106" s="5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B106" s="5" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C106" s="6" t="n">
-        <v>43603</v>
+        <v>44464</v>
       </c>
       <c r="D106" s="6" t="n">
-        <v>43604</v>
+        <v>44465</v>
       </c>
       <c r="E106" s="7" t="s">
         <v>18</v>
@@ -4290,36 +4286,36 @@
         <v>17</v>
       </c>
       <c r="N106" s="8" t="n">
-        <v>44446</v>
+        <v>44445</v>
       </c>
       <c r="O106" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P106" s="8" t="n">
-        <v>44764.6144791667</v>
+        <v>44764.5626388889</v>
       </c>
     </row>
     <row r="107" customHeight="1" ht="20">
       <c r="A107" s="5" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B107" s="5" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C107" s="6" t="n">
-        <v>43506</v>
+        <v>44474</v>
       </c>
       <c r="D107" s="6" t="n">
-        <v>43506</v>
+        <v>44475</v>
       </c>
       <c r="E107" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F107" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="G107" s="5" t="n">
         <v>130</v>
-      </c>
-      <c r="G107" s="5" t="n">
-        <v>30</v>
       </c>
       <c r="H107" s="5"/>
       <c r="I107" s="5"/>
@@ -4330,36 +4326,36 @@
         <v>17</v>
       </c>
       <c r="N107" s="8" t="n">
-        <v>44446</v>
+        <v>44446.2805902778</v>
       </c>
       <c r="O107" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P107" s="8" t="n">
-        <v>44767.5292824074</v>
+        <v>44586.645775463</v>
       </c>
     </row>
     <row r="108" customHeight="1" ht="20">
       <c r="A108" s="5" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B108" s="5" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C108" s="6" t="n">
-        <v>43877</v>
+        <v>43603</v>
       </c>
       <c r="D108" s="6" t="n">
-        <v>43877</v>
+        <v>43604</v>
       </c>
       <c r="E108" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F108" s="5" t="n">
+        <v>230</v>
+      </c>
+      <c r="G108" s="5" t="n">
         <v>130</v>
-      </c>
-      <c r="G108" s="5" t="n">
-        <v>30</v>
       </c>
       <c r="H108" s="5"/>
       <c r="I108" s="5"/>
@@ -4376,30 +4372,30 @@
         <v>17</v>
       </c>
       <c r="P108" s="8" t="n">
-        <v>44767.5397337963</v>
+        <v>44764.6144791667</v>
       </c>
     </row>
     <row r="109" customHeight="1" ht="20">
       <c r="A109" s="5" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B109" s="5" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C109" s="6" t="n">
-        <v>44170</v>
+        <v>43506</v>
       </c>
       <c r="D109" s="6" t="n">
-        <v>44173</v>
+        <v>43506</v>
       </c>
       <c r="E109" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F109" s="5" t="n">
-        <v>495</v>
+        <v>130</v>
       </c>
       <c r="G109" s="5" t="n">
-        <v>310</v>
+        <v>30</v>
       </c>
       <c r="H109" s="5"/>
       <c r="I109" s="5"/>
@@ -4410,32 +4406,36 @@
         <v>17</v>
       </c>
       <c r="N109" s="8" t="n">
-        <v>44446.5258333333</v>
-      </c>
-      <c r="O109" s="7"/>
-      <c r="P109" s="8"/>
+        <v>44446</v>
+      </c>
+      <c r="O109" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P109" s="8" t="n">
+        <v>44767.5292824074</v>
+      </c>
     </row>
     <row r="110" customHeight="1" ht="20">
       <c r="A110" s="5" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B110" s="5" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C110" s="6" t="n">
-        <v>44331</v>
+        <v>43877</v>
       </c>
       <c r="D110" s="6" t="n">
-        <v>44332</v>
+        <v>43877</v>
       </c>
       <c r="E110" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F110" s="5" t="n">
-        <v>230</v>
+        <v>130</v>
       </c>
       <c r="G110" s="5" t="n">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="H110" s="5"/>
       <c r="I110" s="5"/>
@@ -4452,30 +4452,30 @@
         <v>17</v>
       </c>
       <c r="P110" s="8" t="n">
-        <v>44785.5036921296</v>
+        <v>44767.5397337963</v>
       </c>
     </row>
     <row r="111" customHeight="1" ht="20">
       <c r="A111" s="5" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B111" s="5" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C111" s="6" t="n">
-        <v>43554</v>
+        <v>44170</v>
       </c>
       <c r="D111" s="6" t="n">
-        <v>43554</v>
+        <v>44173</v>
       </c>
       <c r="E111" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F111" s="5" t="n">
-        <v>130</v>
+        <v>495</v>
       </c>
       <c r="G111" s="5" t="n">
-        <v>30</v>
+        <v>310</v>
       </c>
       <c r="H111" s="5"/>
       <c r="I111" s="5"/>
@@ -4486,27 +4486,23 @@
         <v>17</v>
       </c>
       <c r="N111" s="8" t="n">
-        <v>44446</v>
-      </c>
-      <c r="O111" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P111" s="8" t="n">
-        <v>44785.5278240741</v>
-      </c>
+        <v>44446.5258333333</v>
+      </c>
+      <c r="O111" s="7"/>
+      <c r="P111" s="8"/>
     </row>
     <row r="112" customHeight="1" ht="20">
       <c r="A112" s="5" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B112" s="5" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C112" s="6" t="n">
-        <v>43764</v>
+        <v>44331</v>
       </c>
       <c r="D112" s="6" t="n">
-        <v>43765</v>
+        <v>44332</v>
       </c>
       <c r="E112" s="7" t="s">
         <v>18</v>
@@ -4532,30 +4528,30 @@
         <v>17</v>
       </c>
       <c r="P112" s="8" t="n">
-        <v>44785.5824074074</v>
+        <v>44785.5036921296</v>
       </c>
     </row>
     <row r="113" customHeight="1" ht="20">
       <c r="A113" s="5" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B113" s="5" t="n">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C113" s="6" t="n">
-        <v>43862</v>
+        <v>43554</v>
       </c>
       <c r="D113" s="6" t="n">
-        <v>43863</v>
+        <v>43554</v>
       </c>
       <c r="E113" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F113" s="5" t="n">
-        <v>230</v>
+        <v>130</v>
       </c>
       <c r="G113" s="5" t="n">
-        <v>130</v>
+        <v>30</v>
       </c>
       <c r="H113" s="5"/>
       <c r="I113" s="5"/>
@@ -4572,7 +4568,7 @@
         <v>17</v>
       </c>
       <c r="P113" s="8" t="n">
-        <v>44785.5965856481</v>
+        <v>44785.5278240741</v>
       </c>
     </row>
     <row r="114" customHeight="1" ht="20">
@@ -4580,13 +4576,13 @@
         <v>48</v>
       </c>
       <c r="B114" s="5" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C114" s="6" t="n">
-        <v>44009</v>
+        <v>43764</v>
       </c>
       <c r="D114" s="6" t="n">
-        <v>44010</v>
+        <v>43765</v>
       </c>
       <c r="E114" s="7" t="s">
         <v>18</v>
@@ -4612,7 +4608,7 @@
         <v>17</v>
       </c>
       <c r="P114" s="8" t="n">
-        <v>44785.6159259259</v>
+        <v>44785.5824074074</v>
       </c>
     </row>
     <row r="115" customHeight="1" ht="20">
@@ -4620,13 +4616,13 @@
         <v>48</v>
       </c>
       <c r="B115" s="5" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C115" s="6" t="n">
-        <v>44100</v>
+        <v>43862</v>
       </c>
       <c r="D115" s="6" t="n">
-        <v>44101</v>
+        <v>43863</v>
       </c>
       <c r="E115" s="7" t="s">
         <v>18</v>
@@ -4652,21 +4648,21 @@
         <v>17</v>
       </c>
       <c r="P115" s="8" t="n">
-        <v>44792.5683217593</v>
+        <v>44785.5965856481</v>
       </c>
     </row>
     <row r="116" customHeight="1" ht="20">
       <c r="A116" s="5" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B116" s="5" t="n">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C116" s="6" t="n">
-        <v>44338</v>
+        <v>44009</v>
       </c>
       <c r="D116" s="6" t="n">
-        <v>44339</v>
+        <v>44010</v>
       </c>
       <c r="E116" s="7" t="s">
         <v>18</v>
@@ -4692,21 +4688,21 @@
         <v>17</v>
       </c>
       <c r="P116" s="8" t="n">
-        <v>44792.5857291667</v>
+        <v>44785.6159259259</v>
       </c>
     </row>
     <row r="117" customHeight="1" ht="20">
       <c r="A117" s="5" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B117" s="5" t="n">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C117" s="6" t="n">
-        <v>44107</v>
+        <v>44100</v>
       </c>
       <c r="D117" s="6" t="n">
-        <v>44108</v>
+        <v>44101</v>
       </c>
       <c r="E117" s="7" t="s">
         <v>18</v>
@@ -4732,21 +4728,21 @@
         <v>17</v>
       </c>
       <c r="P117" s="8" t="n">
-        <v>44819.4365393519</v>
+        <v>44792.5683217593</v>
       </c>
     </row>
     <row r="118" customHeight="1" ht="20">
       <c r="A118" s="5" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B118" s="5" t="n">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C118" s="6" t="n">
-        <v>44401</v>
+        <v>44338</v>
       </c>
       <c r="D118" s="6" t="n">
-        <v>44402</v>
+        <v>44339</v>
       </c>
       <c r="E118" s="7" t="s">
         <v>18</v>
@@ -4772,30 +4768,30 @@
         <v>17</v>
       </c>
       <c r="P118" s="8" t="n">
-        <v>44819.4539351852</v>
+        <v>44792.5857291667</v>
       </c>
     </row>
     <row r="119" customHeight="1" ht="20">
       <c r="A119" s="5" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B119" s="5" t="n">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C119" s="6" t="n">
-        <v>43769</v>
+        <v>44107</v>
       </c>
       <c r="D119" s="6" t="n">
-        <v>43772</v>
+        <v>44108</v>
       </c>
       <c r="E119" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F119" s="5" t="n">
-        <v>495</v>
+        <v>230</v>
       </c>
       <c r="G119" s="5" t="n">
-        <v>245</v>
+        <v>130</v>
       </c>
       <c r="H119" s="5"/>
       <c r="I119" s="5"/>
@@ -4812,30 +4808,30 @@
         <v>17</v>
       </c>
       <c r="P119" s="8" t="n">
-        <v>44819.5838773148</v>
+        <v>44819.4365393519</v>
       </c>
     </row>
     <row r="120" customHeight="1" ht="20">
       <c r="A120" s="5" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B120" s="5" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C120" s="6" t="n">
-        <v>44498</v>
+        <v>44401</v>
       </c>
       <c r="D120" s="6" t="n">
-        <v>44501</v>
+        <v>44402</v>
       </c>
       <c r="E120" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F120" s="5" t="n">
-        <v>495</v>
+        <v>230</v>
       </c>
       <c r="G120" s="5" t="n">
-        <v>310</v>
+        <v>130</v>
       </c>
       <c r="H120" s="5"/>
       <c r="I120" s="5"/>
@@ -4852,30 +4848,30 @@
         <v>17</v>
       </c>
       <c r="P120" s="8" t="n">
-        <v>44837.6617939815</v>
+        <v>44819.4539351852</v>
       </c>
     </row>
     <row r="121" customHeight="1" ht="20">
       <c r="A121" s="5" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B121" s="5" t="n">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C121" s="6" t="n">
-        <v>43981</v>
+        <v>43769</v>
       </c>
       <c r="D121" s="6" t="n">
-        <v>43989</v>
+        <v>43772</v>
       </c>
       <c r="E121" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F121" s="5" t="n">
-        <v>1050</v>
+        <v>495</v>
       </c>
       <c r="G121" s="5" t="n">
-        <v>580</v>
+        <v>245</v>
       </c>
       <c r="H121" s="5"/>
       <c r="I121" s="5"/>
@@ -4886,32 +4882,36 @@
         <v>17</v>
       </c>
       <c r="N121" s="8" t="n">
-        <v>44446.5351157407</v>
-      </c>
-      <c r="O121" s="7"/>
-      <c r="P121" s="8"/>
+        <v>44446</v>
+      </c>
+      <c r="O121" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P121" s="8" t="n">
+        <v>44819.5838773148</v>
+      </c>
     </row>
     <row r="122" customHeight="1" ht="20">
       <c r="A122" s="5" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B122" s="5" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C122" s="6" t="n">
-        <v>44450</v>
+        <v>44498</v>
       </c>
       <c r="D122" s="6" t="n">
-        <v>44457</v>
+        <v>44501</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F122" s="5" t="n">
-        <v>970</v>
+        <v>495</v>
       </c>
       <c r="G122" s="5" t="n">
-        <v>690</v>
+        <v>310</v>
       </c>
       <c r="H122" s="5"/>
       <c r="I122" s="5"/>
@@ -4922,32 +4922,36 @@
         <v>17</v>
       </c>
       <c r="N122" s="8" t="n">
-        <v>44446.5361226852</v>
-      </c>
-      <c r="O122" s="7"/>
-      <c r="P122" s="8"/>
+        <v>44446</v>
+      </c>
+      <c r="O122" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P122" s="8" t="n">
+        <v>44837.6617939815</v>
+      </c>
     </row>
     <row r="123" customHeight="1" ht="20">
       <c r="A123" s="5" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="B123" s="5" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C123" s="6" t="n">
-        <v>44023</v>
+        <v>43981</v>
       </c>
       <c r="D123" s="6" t="n">
-        <v>44029</v>
+        <v>43989</v>
       </c>
       <c r="E123" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F123" s="5" t="n">
-        <v>790</v>
+        <v>1050</v>
       </c>
       <c r="G123" s="5" t="n">
-        <v>570</v>
+        <v>580</v>
       </c>
       <c r="H123" s="5"/>
       <c r="I123" s="5"/>
@@ -4958,32 +4962,32 @@
         <v>17</v>
       </c>
       <c r="N123" s="8" t="n">
-        <v>44446.5370138889</v>
+        <v>44446.5351157407</v>
       </c>
       <c r="O123" s="7"/>
       <c r="P123" s="8"/>
     </row>
     <row r="124" customHeight="1" ht="20">
       <c r="A124" s="5" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="B124" s="5" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="C124" s="6" t="n">
-        <v>43575</v>
+        <v>44450</v>
       </c>
       <c r="D124" s="6" t="n">
-        <v>43581</v>
+        <v>44457</v>
       </c>
       <c r="E124" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F124" s="5" t="n">
-        <v>860</v>
+        <v>970</v>
       </c>
       <c r="G124" s="5" t="n">
-        <v>550</v>
+        <v>690</v>
       </c>
       <c r="H124" s="5"/>
       <c r="I124" s="5"/>
@@ -4994,32 +4998,32 @@
         <v>17</v>
       </c>
       <c r="N124" s="8" t="n">
-        <v>44446.5379398148</v>
+        <v>44446.5361226852</v>
       </c>
       <c r="O124" s="7"/>
       <c r="P124" s="8"/>
     </row>
     <row r="125" customHeight="1" ht="20">
       <c r="A125" s="5" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B125" s="5" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C125" s="6" t="n">
-        <v>44284</v>
+        <v>44023</v>
       </c>
       <c r="D125" s="6" t="n">
-        <v>44290</v>
+        <v>44029</v>
       </c>
       <c r="E125" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F125" s="5" t="n">
-        <v>890</v>
+        <v>790</v>
       </c>
       <c r="G125" s="5" t="n">
-        <v>590</v>
+        <v>570</v>
       </c>
       <c r="H125" s="5"/>
       <c r="I125" s="5"/>
@@ -5030,7 +5034,7 @@
         <v>17</v>
       </c>
       <c r="N125" s="8" t="n">
-        <v>44446.5387268519</v>
+        <v>44446.5370138889</v>
       </c>
       <c r="O125" s="7"/>
       <c r="P125" s="8"/>
@@ -5040,22 +5044,22 @@
         <v>25</v>
       </c>
       <c r="B126" s="5" t="n">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C126" s="6" t="n">
-        <v>44665</v>
+        <v>43575</v>
       </c>
       <c r="D126" s="6" t="n">
-        <v>44671</v>
+        <v>43581</v>
       </c>
       <c r="E126" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F126" s="5" t="n">
-        <v>1150</v>
+        <v>860</v>
       </c>
       <c r="G126" s="5" t="n">
-        <v>770</v>
+        <v>550</v>
       </c>
       <c r="H126" s="5"/>
       <c r="I126" s="5"/>
@@ -5066,36 +5070,32 @@
         <v>17</v>
       </c>
       <c r="N126" s="8" t="n">
-        <v>44446</v>
-      </c>
-      <c r="O126" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P126" s="8" t="n">
-        <v>44676.391724537</v>
-      </c>
+        <v>44446.5379398148</v>
+      </c>
+      <c r="O126" s="7"/>
+      <c r="P126" s="8"/>
     </row>
     <row r="127" customHeight="1" ht="20">
       <c r="A127" s="5" t="n">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="B127" s="5" t="n">
-        <v>263</v>
+        <v>77</v>
       </c>
       <c r="C127" s="6" t="n">
-        <v>44653</v>
+        <v>44284</v>
       </c>
       <c r="D127" s="6" t="n">
-        <v>44653</v>
+        <v>44290</v>
       </c>
       <c r="E127" s="7" t="s">
         <v>16</v>
       </c>
       <c r="F127" s="5" t="n">
-        <v>130</v>
+        <v>890</v>
       </c>
       <c r="G127" s="5" t="n">
-        <v>30</v>
+        <v>590</v>
       </c>
       <c r="H127" s="5"/>
       <c r="I127" s="5"/>
@@ -5106,32 +5106,32 @@
         <v>17</v>
       </c>
       <c r="N127" s="8" t="n">
-        <v>44646.3677199074</v>
+        <v>44446.5387268519</v>
       </c>
       <c r="O127" s="7"/>
       <c r="P127" s="8"/>
     </row>
     <row r="128" customHeight="1" ht="20">
       <c r="A128" s="5" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B128" s="5" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="C128" s="6" t="n">
-        <v>44359</v>
+        <v>44665</v>
       </c>
       <c r="D128" s="6" t="n">
-        <v>44360</v>
+        <v>44671</v>
       </c>
       <c r="E128" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F128" s="5" t="n">
-        <v>230</v>
+        <v>1150</v>
       </c>
       <c r="G128" s="5" t="n">
-        <v>130</v>
+        <v>770</v>
       </c>
       <c r="H128" s="5"/>
       <c r="I128" s="5"/>
@@ -5142,74 +5142,72 @@
         <v>17</v>
       </c>
       <c r="N128" s="8" t="n">
-        <v>44446.542337963</v>
-      </c>
-      <c r="O128" s="7"/>
-      <c r="P128" s="8"/>
+        <v>44446</v>
+      </c>
+      <c r="O128" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P128" s="8" t="n">
+        <v>44676.391724537</v>
+      </c>
     </row>
     <row r="129" customHeight="1" ht="20">
       <c r="A129" s="5" t="n">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="B129" s="5" t="n">
-        <v>85</v>
+        <v>263</v>
       </c>
       <c r="C129" s="6" t="n">
-        <v>44450</v>
+        <v>44653</v>
       </c>
       <c r="D129" s="6" t="n">
-        <v>44453</v>
+        <v>44653</v>
       </c>
       <c r="E129" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F129" s="5" t="n">
-        <v>830</v>
+        <v>130</v>
       </c>
       <c r="G129" s="5" t="n">
-        <v>500</v>
+        <v>30</v>
       </c>
       <c r="H129" s="5"/>
       <c r="I129" s="5"/>
       <c r="J129" s="5"/>
       <c r="K129" s="5"/>
-      <c r="L129" s="7" t="s">
-        <v>21</v>
-      </c>
+      <c r="L129" s="7"/>
       <c r="M129" s="7" t="s">
         <v>17</v>
       </c>
       <c r="N129" s="8" t="n">
-        <v>44447</v>
-      </c>
-      <c r="O129" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P129" s="8" t="n">
-        <v>44837.6220949074</v>
-      </c>
+        <v>44646.3677199074</v>
+      </c>
+      <c r="O129" s="7"/>
+      <c r="P129" s="8"/>
     </row>
     <row r="130" customHeight="1" ht="20">
       <c r="A130" s="5" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="B130" s="5" t="n">
-        <v>342</v>
+        <v>84</v>
       </c>
       <c r="C130" s="6" t="n">
-        <v>44723</v>
+        <v>44359</v>
       </c>
       <c r="D130" s="6" t="n">
-        <v>44724</v>
+        <v>44360</v>
       </c>
       <c r="E130" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F130" s="5" t="n">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="G130" s="5" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="H130" s="5"/>
       <c r="I130" s="5"/>
@@ -5220,67 +5218,65 @@
         <v>17</v>
       </c>
       <c r="N130" s="8" t="n">
-        <v>44665</v>
-      </c>
-      <c r="O130" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P130" s="8" t="n">
-        <v>44731.4374652778</v>
-      </c>
+        <v>44446.542337963</v>
+      </c>
+      <c r="O130" s="7"/>
+      <c r="P130" s="8"/>
     </row>
     <row r="131" customHeight="1" ht="20">
       <c r="A131" s="5" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B131" s="5" t="n">
-        <v>422</v>
+        <v>85</v>
       </c>
       <c r="C131" s="6" t="n">
-        <v>44828</v>
+        <v>44450</v>
       </c>
       <c r="D131" s="6" t="n">
-        <v>44829</v>
+        <v>44453</v>
       </c>
       <c r="E131" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F131" s="5" t="n">
-        <v>245</v>
+        <v>830</v>
       </c>
       <c r="G131" s="5" t="n">
-        <v>140</v>
+        <v>500</v>
       </c>
       <c r="H131" s="5"/>
       <c r="I131" s="5"/>
       <c r="J131" s="5"/>
       <c r="K131" s="5"/>
-      <c r="L131" s="7"/>
+      <c r="L131" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="M131" s="7" t="s">
         <v>17</v>
       </c>
       <c r="N131" s="8" t="n">
-        <v>44748</v>
+        <v>44447</v>
       </c>
       <c r="O131" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P131" s="8" t="n">
-        <v>44830.3892361111</v>
+        <v>44837.6220949074</v>
       </c>
     </row>
     <row r="132" customHeight="1" ht="20">
       <c r="A132" s="5" t="n">
-        <v>181</v>
+        <v>54</v>
       </c>
       <c r="B132" s="5" t="n">
-        <v>502</v>
+        <v>342</v>
       </c>
       <c r="C132" s="6" t="n">
-        <v>44849</v>
+        <v>44723</v>
       </c>
       <c r="D132" s="6" t="n">
-        <v>44850</v>
+        <v>44724</v>
       </c>
       <c r="E132" s="7" t="s">
         <v>18</v>
@@ -5300,13 +5296,13 @@
         <v>17</v>
       </c>
       <c r="N132" s="8" t="n">
-        <v>44810</v>
+        <v>44665</v>
       </c>
       <c r="O132" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P132" s="8" t="n">
-        <v>44847.397962963</v>
+        <v>44731.4374652778</v>
       </c>
     </row>
     <row r="133" customHeight="1" ht="20">
@@ -5314,22 +5310,22 @@
         <v>48</v>
       </c>
       <c r="B133" s="5" t="n">
-        <v>682</v>
+        <v>422</v>
       </c>
       <c r="C133" s="6" t="n">
-        <v>44989</v>
+        <v>44828</v>
       </c>
       <c r="D133" s="6" t="n">
-        <v>44990</v>
+        <v>44829</v>
       </c>
       <c r="E133" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F133" s="5" t="n">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="G133" s="5" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="H133" s="5"/>
       <c r="I133" s="5"/>
@@ -5340,36 +5336,36 @@
         <v>17</v>
       </c>
       <c r="N133" s="8" t="n">
-        <v>44970</v>
+        <v>44748</v>
       </c>
       <c r="O133" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P133" s="8" t="n">
-        <v>44988.7055555556</v>
+        <v>44830.3892361111</v>
       </c>
     </row>
     <row r="134" customHeight="1" ht="20">
       <c r="A134" s="5" t="n">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="B134" s="5" t="n">
-        <v>702</v>
+        <v>502</v>
       </c>
       <c r="C134" s="6" t="n">
-        <v>44996</v>
+        <v>44849</v>
       </c>
       <c r="D134" s="6" t="n">
-        <v>44997</v>
+        <v>44850</v>
       </c>
       <c r="E134" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F134" s="5" t="n">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="G134" s="5" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="H134" s="5"/>
       <c r="I134" s="5"/>
@@ -5380,36 +5376,36 @@
         <v>17</v>
       </c>
       <c r="N134" s="8" t="n">
-        <v>44986</v>
+        <v>44810</v>
       </c>
       <c r="O134" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P134" s="8" t="n">
-        <v>44998.346400463</v>
+        <v>44847.397962963</v>
       </c>
     </row>
     <row r="135" customHeight="1" ht="20">
       <c r="A135" s="5" t="n">
-        <v>281</v>
+        <v>48</v>
       </c>
       <c r="B135" s="5" t="n">
-        <v>822</v>
+        <v>682</v>
       </c>
       <c r="C135" s="6" t="n">
-        <v>45227</v>
+        <v>44989</v>
       </c>
       <c r="D135" s="6" t="n">
-        <v>45230</v>
+        <v>44990</v>
       </c>
       <c r="E135" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F135" s="5" t="n">
-        <v>540</v>
+        <v>250</v>
       </c>
       <c r="G135" s="5" t="n">
-        <v>345</v>
+        <v>150</v>
       </c>
       <c r="H135" s="5"/>
       <c r="I135" s="5"/>
@@ -5420,36 +5416,36 @@
         <v>17</v>
       </c>
       <c r="N135" s="8" t="n">
-        <v>45032</v>
+        <v>44970</v>
       </c>
       <c r="O135" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P135" s="8" t="n">
-        <v>45231.536724537</v>
+        <v>44988.7055555556</v>
       </c>
     </row>
     <row r="136" customHeight="1" ht="20">
       <c r="A136" s="5" t="n">
-        <v>361</v>
+        <v>81</v>
       </c>
       <c r="B136" s="5" t="n">
-        <v>902</v>
+        <v>702</v>
       </c>
       <c r="C136" s="6" t="n">
-        <v>45074</v>
+        <v>44996</v>
       </c>
       <c r="D136" s="6" t="n">
-        <v>45078</v>
+        <v>44997</v>
       </c>
       <c r="E136" s="7" t="s">
         <v>18</v>
       </c>
       <c r="F136" s="5" t="n">
-        <v>695</v>
+        <v>250</v>
       </c>
       <c r="G136" s="5" t="n">
-        <v>495</v>
+        <v>150</v>
       </c>
       <c r="H136" s="5"/>
       <c r="I136" s="5"/>
@@ -5460,36 +5456,36 @@
         <v>17</v>
       </c>
       <c r="N136" s="8" t="n">
-        <v>45069</v>
+        <v>44986</v>
       </c>
       <c r="O136" s="7" t="s">
         <v>17</v>
       </c>
       <c r="P136" s="8" t="n">
-        <v>45071.3412962963</v>
+        <v>44998.346400463</v>
       </c>
     </row>
     <row r="137" customHeight="1" ht="20">
       <c r="A137" s="5" t="n">
-        <v>401</v>
+        <v>281</v>
       </c>
       <c r="B137" s="5" t="n">
-        <v>982</v>
+        <v>822</v>
       </c>
       <c r="C137" s="6" t="n">
-        <v>45129</v>
+        <v>45227</v>
       </c>
       <c r="D137" s="6" t="n">
-        <v>45132</v>
+        <v>45230</v>
       </c>
       <c r="E137" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F137" s="5" t="n">
-        <v>670</v>
+        <v>540</v>
       </c>
       <c r="G137" s="5" t="n">
-        <v>380</v>
+        <v>345</v>
       </c>
       <c r="H137" s="5"/>
       <c r="I137" s="5"/>
@@ -5500,32 +5496,36 @@
         <v>17</v>
       </c>
       <c r="N137" s="8" t="n">
-        <v>45111.2535763889</v>
-      </c>
-      <c r="O137" s="7"/>
-      <c r="P137" s="8"/>
+        <v>45032</v>
+      </c>
+      <c r="O137" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P137" s="8" t="n">
+        <v>45231.536724537</v>
+      </c>
     </row>
     <row r="138" customHeight="1" ht="20">
       <c r="A138" s="5" t="n">
-        <v>41</v>
+        <v>361</v>
       </c>
       <c r="B138" s="5" t="n">
-        <v>1062</v>
+        <v>902</v>
       </c>
       <c r="C138" s="6" t="n">
-        <v>45206</v>
+        <v>45074</v>
       </c>
       <c r="D138" s="6" t="n">
-        <v>45214</v>
+        <v>45078</v>
       </c>
       <c r="E138" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F138" s="5" t="n">
-        <v>1100</v>
+        <v>695</v>
       </c>
       <c r="G138" s="5" t="n">
-        <v>710</v>
+        <v>495</v>
       </c>
       <c r="H138" s="5"/>
       <c r="I138" s="5"/>
@@ -5536,32 +5536,36 @@
         <v>17</v>
       </c>
       <c r="N138" s="8" t="n">
-        <v>45171.606875</v>
-      </c>
-      <c r="O138" s="7"/>
-      <c r="P138" s="8"/>
+        <v>45069</v>
+      </c>
+      <c r="O138" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P138" s="8" t="n">
+        <v>45071.3412962963</v>
+      </c>
     </row>
     <row r="139" customHeight="1" ht="20">
       <c r="A139" s="5" t="n">
-        <v>461</v>
+        <v>401</v>
       </c>
       <c r="B139" s="5" t="n">
-        <v>1302</v>
+        <v>982</v>
       </c>
       <c r="C139" s="6" t="n">
-        <v>45346</v>
+        <v>45129</v>
       </c>
       <c r="D139" s="6" t="n">
-        <v>45347</v>
+        <v>45132</v>
       </c>
       <c r="E139" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F139" s="5" t="n">
-        <v>250</v>
+        <v>670</v>
       </c>
       <c r="G139" s="5" t="n">
-        <v>150</v>
+        <v>380</v>
       </c>
       <c r="H139" s="5"/>
       <c r="I139" s="5"/>
@@ -5572,36 +5576,32 @@
         <v>17</v>
       </c>
       <c r="N139" s="8" t="n">
-        <v>45308</v>
-      </c>
-      <c r="O139" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="P139" s="8" t="n">
-        <v>45345.4013194444</v>
-      </c>
+        <v>45111.2535763889</v>
+      </c>
+      <c r="O139" s="7"/>
+      <c r="P139" s="8"/>
     </row>
     <row r="140" customHeight="1" ht="20">
       <c r="A140" s="5" t="n">
-        <v>541</v>
+        <v>41</v>
       </c>
       <c r="B140" s="5" t="n">
-        <v>1503</v>
+        <v>1062</v>
       </c>
       <c r="C140" s="6" t="n">
-        <v>45594</v>
+        <v>45206</v>
       </c>
       <c r="D140" s="6" t="n">
-        <v>45598</v>
+        <v>45214</v>
       </c>
       <c r="E140" s="7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F140" s="5" t="n">
-        <v>690</v>
+        <v>1100</v>
       </c>
       <c r="G140" s="5" t="n">
-        <v>690</v>
+        <v>710</v>
       </c>
       <c r="H140" s="5"/>
       <c r="I140" s="5"/>
@@ -5609,39 +5609,35 @@
       <c r="K140" s="5"/>
       <c r="L140" s="7"/>
       <c r="M140" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="N140" s="8" t="n">
-        <v>45582</v>
-      </c>
-      <c r="O140" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="P140" s="8" t="n">
-        <v>45793.6943287037</v>
-      </c>
+        <v>45171.606875</v>
+      </c>
+      <c r="O140" s="7"/>
+      <c r="P140" s="8"/>
     </row>
     <row r="141" customHeight="1" ht="20">
       <c r="A141" s="5" t="n">
-        <v>821</v>
+        <v>461</v>
       </c>
       <c r="B141" s="5" t="n">
-        <v>1783</v>
+        <v>1302</v>
       </c>
       <c r="C141" s="6" t="n">
-        <v>45996</v>
+        <v>45346</v>
       </c>
       <c r="D141" s="6" t="n">
-        <v>45998</v>
+        <v>45347</v>
       </c>
       <c r="E141" s="7" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F141" s="5" t="n">
-        <v>490</v>
+        <v>250</v>
       </c>
       <c r="G141" s="5" t="n">
-        <v>490</v>
+        <v>150</v>
       </c>
       <c r="H141" s="5"/>
       <c r="I141" s="5"/>
@@ -5649,26 +5645,30 @@
       <c r="K141" s="5"/>
       <c r="L141" s="7"/>
       <c r="M141" s="7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="N141" s="8" t="n">
-        <v>45983.3458449074</v>
-      </c>
-      <c r="O141" s="7"/>
-      <c r="P141" s="8"/>
+        <v>45308</v>
+      </c>
+      <c r="O141" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="P141" s="8" t="n">
+        <v>45345.4013194444</v>
+      </c>
     </row>
     <row r="142" customHeight="1" ht="20">
       <c r="A142" s="5" t="n">
         <v>541</v>
       </c>
       <c r="B142" s="5" t="n">
-        <v>1664</v>
+        <v>1503</v>
       </c>
       <c r="C142" s="6" t="n">
-        <v>45915</v>
+        <v>45594</v>
       </c>
       <c r="D142" s="6" t="n">
-        <v>45919</v>
+        <v>45598</v>
       </c>
       <c r="E142" s="7" t="s">
         <v>18</v>
@@ -5688,12 +5688,88 @@
         <v>19</v>
       </c>
       <c r="N142" s="8" t="n">
-        <v>45811</v>
+        <v>45582</v>
       </c>
       <c r="O142" s="7" t="s">
         <v>19</v>
       </c>
       <c r="P142" s="8" t="n">
+        <v>45793.6943287037</v>
+      </c>
+    </row>
+    <row r="143" customHeight="1" ht="20">
+      <c r="A143" s="5" t="n">
+        <v>821</v>
+      </c>
+      <c r="B143" s="5" t="n">
+        <v>1783</v>
+      </c>
+      <c r="C143" s="6" t="n">
+        <v>45996</v>
+      </c>
+      <c r="D143" s="6" t="n">
+        <v>45998</v>
+      </c>
+      <c r="E143" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F143" s="5" t="n">
+        <v>490</v>
+      </c>
+      <c r="G143" s="5" t="n">
+        <v>490</v>
+      </c>
+      <c r="H143" s="5"/>
+      <c r="I143" s="5"/>
+      <c r="J143" s="5"/>
+      <c r="K143" s="5"/>
+      <c r="L143" s="7"/>
+      <c r="M143" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="N143" s="8" t="n">
+        <v>45983.3458449074</v>
+      </c>
+      <c r="O143" s="7"/>
+      <c r="P143" s="8"/>
+    </row>
+    <row r="144" customHeight="1" ht="20">
+      <c r="A144" s="5" t="n">
+        <v>541</v>
+      </c>
+      <c r="B144" s="5" t="n">
+        <v>1664</v>
+      </c>
+      <c r="C144" s="6" t="n">
+        <v>45915</v>
+      </c>
+      <c r="D144" s="6" t="n">
+        <v>45919</v>
+      </c>
+      <c r="E144" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F144" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="G144" s="5" t="n">
+        <v>690</v>
+      </c>
+      <c r="H144" s="5"/>
+      <c r="I144" s="5"/>
+      <c r="J144" s="5"/>
+      <c r="K144" s="5"/>
+      <c r="L144" s="7"/>
+      <c r="M144" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="N144" s="8" t="n">
+        <v>45811</v>
+      </c>
+      <c r="O144" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="P144" s="8" t="n">
         <v>45951.6466550926</v>
       </c>
     </row>

</xml_diff>